<commit_message>
feat: Update Automation Projects Status.xlsx with new data
</commit_message>
<xml_diff>
--- a/Ansible to Orchestrator Transition/Automation Projects Status.xlsx
+++ b/Ansible to Orchestrator Transition/Automation Projects Status.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\GitHub-LocalRepos\AutomationProjects\Ansible to Orchestrator Transition\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F444274-7253-47F1-9C58-E12CFE4C2955}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C13254F-63C4-4765-9D94-BDC257A8D969}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10125" yWindow="1725" windowWidth="41340" windowHeight="17445" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="19">
   <si>
     <t>Rank</t>
   </si>
@@ -84,6 +84,15 @@
   </si>
   <si>
     <t>Automation code packaged and imported into CVS-DEV VCF Instance.  Documentation placed in Broadcom Teams share</t>
+  </si>
+  <si>
+    <t>Service Accounts Report</t>
+  </si>
+  <si>
+    <t>Get Datastores 75% to 100% used</t>
+  </si>
+  <si>
+    <t>Automation code packaged and imported into CVS-DEV VCF Instance.  Documentation emailed to Jevonnah</t>
   </si>
 </sst>
 </file>
@@ -489,7 +498,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="2"/>
@@ -580,6 +589,9 @@
       <c r="D5" t="s">
         <v>12</v>
       </c>
+      <c r="E5" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
@@ -610,6 +622,40 @@
       </c>
       <c r="E7" t="s">
         <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="2">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="D8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="2">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="D9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E9" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -627,12 +673,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100F31F3E2BDF57D84FBD1940DB5BFE70A1" ma:contentTypeVersion="7" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="a9b561b9de271dadfdbb55af4b004760">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="214119f6-a8cf-4ab0-bc74-24d72ad44cda" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9d4541ef4acfa0f2fee95c92c0176a78" ns2:_="">
     <xsd:import namespace="214119f6-a8cf-4ab0-bc74-24d72ad44cda"/>
@@ -794,6 +834,12 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{542E298F-43A9-4446-A1AB-E11718AE2464}">
   <ds:schemaRefs>
@@ -803,15 +849,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{057DAA1B-1D4D-4A47-8C00-D92C3521D8BF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CB283DE-2B0E-40C6-AE8D-C954DDF5DDF4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -827,4 +864,13 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{057DAA1B-1D4D-4A47-8C00-D92C3521D8BF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Add service account expiration reporting scripts and tests
- Introduced gen-awkward.js to generate invocation strings for testing PowerShell script execution.
- Created test-action.js to validate the behavior of buildServiceAccountExpirationInvocation.js with various input scenarios.
- Added test-workflow-tasks.js to ensure the integrity of task code within Get-ServiceAccountExpirationReport_spec.js.
- Implemented service_accounts_report.yml playbook for executing PowerShell scripts remotely via Ansible.
- Defined variables in vars.txt for configurable parameters used in the playbook.
</commit_message>
<xml_diff>
--- a/Ansible to Orchestrator Transition/Automation Projects Status.xlsx
+++ b/Ansible to Orchestrator Transition/Automation Projects Status.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\GitHub-LocalRepos\AutomationProjects\Ansible to Orchestrator Transition\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B43645F-0E25-4544-B123-4C9572949A34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E50297BB-5540-4DE7-BD0C-F8A7BF671D8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5070" yWindow="5070" windowWidth="38700" windowHeight="15435" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4680" yWindow="4140" windowWidth="30075" windowHeight="13095" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -621,7 +621,10 @@
         <v>6</v>
       </c>
       <c r="D7" t="s">
-        <v>7</v>
+        <v>12</v>
+      </c>
+      <c r="E7" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -635,10 +638,7 @@
         <v>6</v>
       </c>
       <c r="D8" t="s">
-        <v>10</v>
-      </c>
-      <c r="E8" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -664,6 +664,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100F31F3E2BDF57D84FBD1940DB5BFE70A1" ma:contentTypeVersion="7" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="a9b561b9de271dadfdbb55af4b004760">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="214119f6-a8cf-4ab0-bc74-24d72ad44cda" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9d4541ef4acfa0f2fee95c92c0176a78" ns2:_="">
     <xsd:import namespace="214119f6-a8cf-4ab0-bc74-24d72ad44cda"/>
@@ -825,15 +834,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement/>
@@ -841,6 +841,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{542E298F-43A9-4446-A1AB-E11718AE2464}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CB283DE-2B0E-40C6-AE8D-C954DDF5DDF4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -858,14 +866,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{542E298F-43A9-4446-A1AB-E11718AE2464}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{057DAA1B-1D4D-4A47-8C00-D92C3521D8BF}">
   <ds:schemaRefs>

</xml_diff>